<commit_message>
spawns sub-agents for each section of CV
</commit_message>
<xml_diff>
--- a/cv-outputs/applications_tracker.xlsx
+++ b/cv-outputs/applications_tracker.xlsx
@@ -1,115 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\CV_crawl\cv-outputs\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_57B1D3DC116CAA5FED5B449649FCB639D4F4D6C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Applications" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Applications" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
-  <si>
-    <t>Date Applied</t>
-  </si>
-  <si>
-    <t>Company</t>
-  </si>
-  <si>
-    <t>Job Title</t>
-  </si>
-  <si>
-    <t>City</t>
-  </si>
-  <si>
-    <t>Job Description</t>
-  </si>
-  <si>
-    <t>Job URL</t>
-  </si>
-  <si>
-    <t>2026-03-19</t>
-  </si>
-  <si>
-    <t>Northslope Technologies</t>
-  </si>
-  <si>
-    <t>Forward Deployed Software Engineer</t>
-  </si>
-  <si>
-    <t>New York, United States</t>
-  </si>
-  <si>
-    <t>Northslope builds customized AI reasoning systems. As a Forward Deployed Software Engineer you will help customers solve their most valuable problems, working closely with stakeholders to conceive, architect, build, and maintain applications. You'll understand a customer's most critical objectives and build operationalized workflows on their enterprise data. Required: Python/TypeScript, production environment experience, end-to-end solutions, structured and unstructured data. Nice to have: Palantir Foundry, React, Spark, LLM-based solutions.</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/jobs/view/4218796460</t>
-  </si>
-  <si>
-    <t>2026-03-23</t>
-  </si>
-  <si>
-    <t>Nira Energy</t>
-  </si>
-  <si>
-    <t>Forward Deployed Engineer</t>
-  </si>
-  <si>
-    <t>New York City, NY (Hybrid/Remote)</t>
-  </si>
-  <si>
-    <t>Nira Energy's mission is to help convert the US power grid to be 100% fossil-free. As the first Forward Deployed Engineer, you'll launch Nira's new business line with Independent System Operators (ISOs). Strong coding skills with 2+ years software engineering experience required. Salary: \90,000-\10,000 with equity.</t>
-  </si>
-  <si>
-    <t>https://job-boards.greenhouse.io/niraenergy/jobs/4964468008</t>
-  </si>
-  <si>
-    <t>2026-03-24</t>
-  </si>
-  <si>
-    <t>Cohere</t>
-  </si>
-  <si>
-    <t>Forward Deployed Engineer, Prompt Specialist</t>
-  </si>
-  <si>
-    <t>Toronto, Ontario, Canada</t>
-  </si>
-  <si>
-    <t>Who are we? Our mission is to scale intelligence to serve humanity. We're training and deploying frontier models for developers and enterprises who are building AI systems to power magical experiences like content generation, semantic search, RAG, and agents. We believe that our work is instrumental to the widespread adoption of AI.</t>
-  </si>
-  <si>
-    <t>https://jobs.ashbyhq.com/cohere/6745547c-cc72-466c-867c-a0539b04909b</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -128,21 +46,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -430,95 +407,180 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="46" customWidth="1"/>
-    <col min="4" max="4" width="35" customWidth="1"/>
-    <col min="5" max="6" width="60" customWidth="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="6"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Date Applied</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Job Title</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Job URL</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" t="s">
-        <v>11</v>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Northslope Technologies</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Forward Deployed Software Engineer</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>New York, United States</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Northslope builds customized AI reasoning systems. As a Forward Deployed Software Engineer you will help customers solve their most valuable problems, working closely with stakeholders to conceive, architect, build, and maintain applications. You'll understand a customer's most critical objectives and build operationalized workflows on their enterprise data. Required: Python/TypeScript, production environment experience, end-to-end solutions, structured and unstructured data. Nice to have: Palantir Foundry, React, Spark, LLM-based solutions.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4218796460</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" t="s">
-        <v>17</v>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Nira Energy</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Forward Deployed Engineer</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>New York City, NY (Hybrid/Remote)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Nira Energy's mission is to help convert the US power grid to be 100% fossil-free. As the first Forward Deployed Engineer, you'll launch Nira's new business line with Independent System Operators (ISOs). Strong coding skills with 2+ years software engineering experience required. Salary: \90,000-\10,000 with equity.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/niraenergy/jobs/4964468008</t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" t="s">
-        <v>23</v>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Cohere</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Forward Deployed Engineer, Prompt Specialist</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Toronto, Ontario, Canada</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Who are we? Our mission is to scale intelligence to serve humanity. We're training and deploying frontier models for developers and enterprises who are building AI systems to power magical experiences like content generation, semantic search, RAG, and agents. We believe that our work is instrumental to the widespread adoption of AI.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/cohere/6745547c-cc72-466c-867c-a0539b04909b</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ElevenLabs</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Forward Deployed Engineer - Strategist</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>About Eleven Labs Eleven Labs is an AI research and product company transforming how we interact with technology. We launched in January 2023 with the first human-like AI voice model. Today, we serve millions of users and thousands of businesses - from fast-growing startups to large enterprises like Deutsche Telekom and Meta. Our investors are some of the world's most prominent, including Andreessen Horowitz, ICONIQ Growth and Sequoia. We've raised $781M in funding and our last valuation was $11B - multiples of 11, always. We have expanded from voice into three main platforms: Eleven Agents enables businesses to deliver seamless and intelligent customer experiences, with the integrations, testing, monitoring, and reliability necessary to deploy voice and chat agents at scale. Eleven Creative empowers creators and marketers to generate and edit speech, music, image, and video across 70+ languages. Eleven API gives developers access to our leading AI audio foundational models. Everything we do is the result of the creativity and commitment of our team - builders doing the best work of their lives. We are researchers, engineers, and operators. IOI medalists and ex-founders. If you want to work hard and create lasting positive impact, we want to hear from you. How we work High-velocity: Rapid experimentation, lean autonomous teams, and minimal bureaucracy. Impact not job titles: We don’t have job titles. Instead, it’s about the impact you have. No task is above or beneath you. AI first: We use AI to move faster with higher-quality results. We do this across the whole company—from engineering to growth to operations. Excellence everywhere: Everything we do should match the quality of our AI models. Global team: We prioritize your talent, not your location. What we offer Innovative culture: You’ll be part of a generational opportunity to define the trajectory of AI, surrounded by a team pushing the boundaries of what’s possible. Growth paths: Joining Eleven Labs</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/elevenlabs/8c068ebf-c79f-4f12-97ef-b4c9a4f7ae5f</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>